<commit_message>
Full spinup procedure with OUT at every loop - done and tested
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/restart_broken/RESTART.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/restart_broken/RESTART.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\automatic_loops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\restart_broken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8854239-FFBB-4960-BA41-EC552E46B877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D71CDC4-F029-4C7F-ADCF-F9DEE3A35F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="43">
   <si>
     <t>-------------------</t>
   </si>
@@ -160,9 +160,6 @@
   </si>
   <si>
     <t>regridded</t>
-  </si>
-  <si>
-    <t>snow_all</t>
   </si>
   <si>
     <t>all_lateral</t>
@@ -633,7 +630,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>24</v>
@@ -889,9 +886,6 @@
     <row r="38" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.35">

</xml_diff>